<commit_message>
Update Excel template with revised form (v1.6.26)
</commit_message>
<xml_diff>
--- a/app/src/main/assets/lib/template.xlsx
+++ b/app/src/main/assets/lib/template.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://skydrive3m-my.sharepoint.com/personal/kr002531_mmm_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KR002531\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{E545C069-09B8-4326-A40C-8B1BF1CAF8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84A2FB46-A4C1-4D61-B046-B45300C01B95}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1543A8-7F8C-4DD8-8097-D33E8AF1979C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{E55886AB-E20E-4A2C-88BD-EDD2C06AAD55}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E55886AB-E20E-4A2C-88BD-EDD2C06AAD55}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="5" r:id="rId1"/>
     <sheet name="비용내역" sheetId="2" r:id="rId2"/>
     <sheet name="행사사진" sheetId="3" r:id="rId3"/>
-    <sheet name="영수증" sheetId="4" r:id="rId4"/>
+    <sheet name="영수증" sheetId="7" r:id="rId4"/>
     <sheet name="Global ID" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Global ID'!$A$1:$D$1316</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2680" uniqueCount="2631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2673" uniqueCount="2630">
   <si>
     <t>정회원 참석자</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -7993,6 +7993,22 @@
   <si>
     <t>이진호(2)</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>법인카드 영수증 - 지원금&gt;</t>
+    </r>
   </si>
   <si>
     <r>
@@ -8009,27 +8025,6 @@
       </rPr>
       <t>개인카드 영수증 - 자부담&gt;</t>
     </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>&lt;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>법인카드 영수증 - 지원금&gt;</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>행사비</t>
   </si>
 </sst>
 </file>
@@ -8325,7 +8320,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -8461,15 +8456,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -8484,6 +8470,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -8905,8 +8897,8 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18">
-      <c r="B2" s="52"/>
-      <c r="C2" s="53"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="50"/>
       <c r="D2" s="4" t="s">
         <v>23</v>
       </c>
@@ -8935,16 +8927,16 @@
       </c>
       <c r="K4" s="9">
         <f>COUNTA(D5:D124)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:18">
       <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="1">
-        <f>_xlfn.XLOOKUP(D5,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>920</v>
+      <c r="C5" s="1" t="str">
+        <f>IF(D5="","",_xlfn.XLOOKUP(D5,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D5" s="23"/>
       <c r="E5" s="2" t="str">
@@ -8959,9 +8951,9 @@
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="1">
-        <f>_xlfn.XLOOKUP(D6,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>3715</v>
+      <c r="C6" s="1" t="str">
+        <f>IF(D6="","",_xlfn.XLOOKUP(D6,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D6" s="23"/>
       <c r="E6" s="2" t="str">
@@ -8976,16 +8968,16 @@
       </c>
       <c r="K6" s="9">
         <f>SUM(G5:G25)</f>
-        <v>300000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:18">
       <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7" s="1">
-        <f>_xlfn.XLOOKUP(D7,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>4672</v>
+      <c r="C7" s="1" t="str">
+        <f>IF(D7="","",_xlfn.XLOOKUP(D7,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D7" s="23"/>
       <c r="E7" s="2" t="str">
@@ -9000,16 +8992,16 @@
       </c>
       <c r="K7" s="9">
         <f>SUMIF($H$5:$H$25,"행사비",$G$5:$G$25)</f>
-        <v>300000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:18">
       <c r="B8" s="1">
         <v>4</v>
       </c>
-      <c r="C8" s="1">
-        <f>_xlfn.XLOOKUP(D8,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>4216</v>
+      <c r="C8" s="1" t="str">
+        <f>IF(D8="","",_xlfn.XLOOKUP(D8,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D8" s="23"/>
       <c r="E8" s="2" t="str">
@@ -9031,9 +9023,9 @@
       <c r="B9" s="1">
         <v>5</v>
       </c>
-      <c r="C9" s="1">
-        <f>_xlfn.XLOOKUP(D9,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>2070</v>
+      <c r="C9" s="1" t="str">
+        <f>IF(D9="","",_xlfn.XLOOKUP(D9,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D9" s="23"/>
       <c r="E9" s="2" t="str">
@@ -9050,11 +9042,11 @@
         <f>SUMIF($H$5:$H$25,"상품",$G$5:$G$25)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="54" t="str">
+      <c r="L9" s="51" t="str">
         <f>IF(K9=0,"",IF(K4&lt;10,"필요 참석자 수 부족. 최소 정회원 10명 이상 참석 시 상품비 사용 가능. 상품비 "&amp;TEXT(K9,"0,0")&amp;"원 전액 행사비에 포함 후 정산",IF((K9+SUM(G30:G34))&gt;500000,"상품비 연 50만원 초과 불가. 총 상품비용 "&amp;TEXT(K9+SUM(G30:G34),"0,0")&amp;"으로, 초과 금액 "&amp;TEXT((K9+SUM(G30:G34))-500000,"0,0")&amp;"원은 행사비에 포함 후 정산","")))</f>
         <v/>
       </c>
-      <c r="M9" s="54"/>
+      <c r="M9" s="51"/>
       <c r="N9" s="26"/>
       <c r="O9" s="26"/>
       <c r="P9" s="26"/>
@@ -9065,9 +9057,9 @@
       <c r="B10" s="1">
         <v>6</v>
       </c>
-      <c r="C10" s="1">
-        <f>_xlfn.XLOOKUP(D10,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C10" s="1" t="str">
+        <f>IF(D10="","",_xlfn.XLOOKUP(D10,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D10" s="23"/>
       <c r="E10" s="2" t="str">
@@ -9082,8 +9074,8 @@
         <v>※ 본 행사 상품비 잔여 한도: 500,000원</v>
       </c>
       <c r="K10" s="18"/>
-      <c r="L10" s="54"/>
-      <c r="M10" s="54"/>
+      <c r="L10" s="51"/>
+      <c r="M10" s="51"/>
       <c r="N10" s="26"/>
       <c r="O10" s="26"/>
       <c r="P10" s="26"/>
@@ -9094,9 +9086,9 @@
       <c r="B11" s="1">
         <v>7</v>
       </c>
-      <c r="C11" s="1">
-        <f>_xlfn.XLOOKUP(D11,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C11" s="1" t="str">
+        <f>IF(D11="","",_xlfn.XLOOKUP(D11,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D11" s="23"/>
       <c r="E11" s="2" t="str">
@@ -9113,9 +9105,9 @@
       <c r="B12" s="1">
         <v>8</v>
       </c>
-      <c r="C12" s="1">
-        <f>_xlfn.XLOOKUP(D12,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C12" s="1" t="str">
+        <f>IF(D12="","",_xlfn.XLOOKUP(D12,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D12" s="23"/>
       <c r="E12" s="2" t="str">
@@ -9128,22 +9120,22 @@
       <c r="J12" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="K12" s="9" cm="1">
+      <c r="K12" s="9" t="str" cm="1">
         <f t="array" ref="K12">IF(K4=0,"",_xlfn.IFS(K4&lt;10,(K7+K9)/K4,K9+SUM(G30:G34)&gt;500000,(K7+(K9+SUM(G30:G34)-500000))/K4,AND(K4&gt;=10,K9+SUM(G30:G34)&lt;=500000),K7/K4))</f>
-        <v>60000</v>
+        <v/>
       </c>
       <c r="L12" s="13" t="str" cm="1">
         <f t="array" ref="L12">IF(K7=0,"",_xlfn.IFS($K$12="","",$K$12&lt;=30000, "전액지원", $K$12&lt;=60000, "20% 자체 부담", $K$12&lt;=120000, "'나' 구간 자부담 비용 + 60,000원 초과 금액에 대해 40% 자체 부담", $K$12&gt;120000, "85,000원 이외 금액 자체 부담(최대 인당 8.5만원 지원)"))</f>
-        <v>20% 자체 부담</v>
+        <v/>
       </c>
     </row>
     <row r="13" spans="2:18">
       <c r="B13" s="1">
         <v>9</v>
       </c>
-      <c r="C13" s="1">
-        <f>_xlfn.XLOOKUP(D13,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C13" s="1" t="str">
+        <f>IF(D13="","",_xlfn.XLOOKUP(D13,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D13" s="23"/>
       <c r="E13" s="2" t="str">
@@ -9159,9 +9151,9 @@
       <c r="B14" s="1">
         <v>10</v>
       </c>
-      <c r="C14" s="1">
-        <f>_xlfn.XLOOKUP(D14,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C14" s="1" t="str">
+        <f>IF(D14="","",_xlfn.XLOOKUP(D14,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D14" s="23"/>
       <c r="E14" s="2" t="str">
@@ -9185,9 +9177,9 @@
       <c r="B15" s="1">
         <v>11</v>
       </c>
-      <c r="C15" s="1">
-        <f>_xlfn.XLOOKUP(D15,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C15" s="1" t="str">
+        <f>IF(D15="","",_xlfn.XLOOKUP(D15,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D15" s="23"/>
       <c r="E15" s="2" t="str">
@@ -9213,9 +9205,9 @@
       <c r="B16" s="1">
         <v>12</v>
       </c>
-      <c r="C16" s="1">
-        <f>_xlfn.XLOOKUP(D16,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C16" s="1" t="str">
+        <f>IF(D16="","",_xlfn.XLOOKUP(D16,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D16" s="23"/>
       <c r="E16" s="2" t="str">
@@ -9230,20 +9222,20 @@
       </c>
       <c r="K16" s="9" cm="1">
         <f t="array" ref="K16">_xlfn.IFS(OR(K12&lt;=30000,K12&gt;120000),0,AND(K12&gt;30000,K12&lt;=60000),K12,K12&gt;60000,60000)</f>
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="L16" s="9">
         <f>K16*20%</f>
-        <v>12000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:18">
       <c r="B17" s="1">
         <v>13</v>
       </c>
-      <c r="C17" s="1">
-        <f>_xlfn.XLOOKUP(D17,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C17" s="1" t="str">
+        <f>IF(D17="","",_xlfn.XLOOKUP(D17,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D17" s="23"/>
       <c r="E17" s="2" t="str">
@@ -9269,9 +9261,9 @@
       <c r="B18" s="1">
         <v>14</v>
       </c>
-      <c r="C18" s="1">
-        <f>_xlfn.XLOOKUP(D18,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C18" s="1" t="str">
+        <f>IF(D18="","",_xlfn.XLOOKUP(D18,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D18" s="23"/>
       <c r="E18" s="2" t="str">
@@ -9284,22 +9276,22 @@
       <c r="J18" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="K18" s="9" cm="1">
+      <c r="K18" s="9" t="str" cm="1">
         <f t="array" ref="K18">_xlfn.IFS(K12&lt;=120000,0,K12&gt;120000,K12)</f>
-        <v>0</v>
-      </c>
-      <c r="L18" s="9">
+        <v/>
+      </c>
+      <c r="L18" s="9" t="str">
         <f>IF(ISERROR(IF(K18=0,0,K18-85000)),"",IF(K18=0,0,K18-85000))</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="19" spans="2:18">
       <c r="B19" s="1">
         <v>15</v>
       </c>
-      <c r="C19" s="1">
-        <f>_xlfn.XLOOKUP(D19,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C19" s="1" t="str">
+        <f>IF(D19="","",_xlfn.XLOOKUP(D19,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D19" s="23"/>
       <c r="E19" s="2" t="str">
@@ -9314,9 +9306,9 @@
       <c r="B20" s="1">
         <v>16</v>
       </c>
-      <c r="C20" s="1">
-        <f>_xlfn.XLOOKUP(D20,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C20" s="1" t="str">
+        <f>IF(D20="","",_xlfn.XLOOKUP(D20,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D20" s="23"/>
       <c r="E20" s="2" t="str">
@@ -9331,7 +9323,7 @@
       </c>
       <c r="K20" s="12">
         <f>SUM(L15:L18)</f>
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="R20" s="6"/>
     </row>
@@ -9339,9 +9331,9 @@
       <c r="B21" s="1">
         <v>17</v>
       </c>
-      <c r="C21" s="1">
-        <f>_xlfn.XLOOKUP(D21,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C21" s="1" t="str">
+        <f>IF(D21="","",_xlfn.XLOOKUP(D21,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D21" s="23"/>
       <c r="E21" s="2" t="str">
@@ -9356,16 +9348,16 @@
       </c>
       <c r="K21" s="12">
         <f>SUM(L15:L18)*K4</f>
-        <v>60000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:18">
       <c r="B22" s="1">
         <v>18</v>
       </c>
-      <c r="C22" s="1">
-        <f>_xlfn.XLOOKUP(D22,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C22" s="1" t="str">
+        <f>IF(D22="","",_xlfn.XLOOKUP(D22,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D22" s="23"/>
       <c r="E22" s="2" t="str">
@@ -9378,18 +9370,18 @@
       <c r="J22" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="K22" s="17">
+      <c r="K22" s="17" t="str">
         <f>IF(ISERROR(K21/K6),"",K21/K6)</f>
-        <v>0.2</v>
+        <v/>
       </c>
     </row>
     <row r="23" spans="2:18">
       <c r="B23" s="1">
         <v>19</v>
       </c>
-      <c r="C23" s="1">
-        <f>_xlfn.XLOOKUP(D23,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C23" s="1" t="str">
+        <f>IF(D23="","",_xlfn.XLOOKUP(D23,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D23" s="23"/>
       <c r="E23" s="2" t="str">
@@ -9404,9 +9396,9 @@
       <c r="B24" s="1">
         <v>20</v>
       </c>
-      <c r="C24" s="1">
-        <f>_xlfn.XLOOKUP(D24,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C24" s="1" t="str">
+        <f>IF(D24="","",_xlfn.XLOOKUP(D24,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D24" s="23"/>
       <c r="E24" s="2" t="str">
@@ -9419,18 +9411,15 @@
       <c r="J24" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="K24" s="31">
-        <f>SUM(L15:L18)*K4</f>
-        <v>0</v>
-      </c>
+      <c r="K24" s="31"/>
     </row>
     <row r="25" spans="2:18">
       <c r="B25" s="1">
         <v>21</v>
       </c>
-      <c r="C25" s="1">
-        <f>_xlfn.XLOOKUP(D25,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C25" s="1" t="str">
+        <f>IF(D25="","",_xlfn.XLOOKUP(D25,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D25" s="23"/>
       <c r="E25" s="2" t="str">
@@ -9443,22 +9432,22 @@
       <c r="J25" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="K25" s="17">
+      <c r="K25" s="17" t="str">
         <f>IF(K24="","",K24/K6)</f>
-        <v>0.20333333333333334</v>
+        <v/>
       </c>
       <c r="L25" s="32" t="str">
         <f>IF(K25="","",IF(K25&gt;=K22,"정산 문제 없음. 최소 자부담 비용보다 "&amp;TEXT(K24-K21,"#,#")&amp;"원 추가 부담함", "최소 자부담 비용 미달. "&amp;TEXT(K21-K24,"#,#")&amp;"원 추가 자부담 필요."))</f>
-        <v>정산 문제 없음. 최소 자부담 비용보다 1,000원 추가 부담함</v>
+        <v/>
       </c>
     </row>
     <row r="26" spans="2:18">
       <c r="B26" s="1">
         <v>22</v>
       </c>
-      <c r="C26" s="1">
-        <f>_xlfn.XLOOKUP(D26,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C26" s="1" t="str">
+        <f>IF(D26="","",_xlfn.XLOOKUP(D26,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D26" s="23"/>
       <c r="E26" s="2" t="str">
@@ -9472,19 +9461,19 @@
       <c r="B27" s="1">
         <v>23</v>
       </c>
-      <c r="C27" s="1">
-        <f>_xlfn.XLOOKUP(D27,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C27" s="1" t="str">
+        <f>IF(D27="","",_xlfn.XLOOKUP(D27,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D27" s="23"/>
       <c r="E27" s="2" t="str">
         <f>IF(NOT(_xlfn.ISFORMULA(C27)),"",IF(D27="","",IF(COUNTIF('Global ID'!$C:$C,D27)&gt;1,"사번확인요","")))</f>
         <v/>
       </c>
-      <c r="F27" s="50" t="s">
+      <c r="F27" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="G27" s="50"/>
+      <c r="G27" s="47"/>
       <c r="K27" s="29"/>
       <c r="L27" s="29"/>
     </row>
@@ -9492,27 +9481,27 @@
       <c r="B28" s="1">
         <v>24</v>
       </c>
-      <c r="C28" s="1">
-        <f>_xlfn.XLOOKUP(D28,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C28" s="1" t="str">
+        <f>IF(D28="","",_xlfn.XLOOKUP(D28,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D28" s="23"/>
       <c r="E28" s="2" t="str">
         <f>IF(NOT(_xlfn.ISFORMULA(C28)),"",IF(D28="","",IF(COUNTIF('Global ID'!$C:$C,D28)&gt;1,"사번확인요","")))</f>
         <v/>
       </c>
-      <c r="F28" s="51" t="s">
+      <c r="F28" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="G28" s="51"/>
+      <c r="G28" s="48"/>
     </row>
     <row r="29" spans="2:18">
       <c r="B29" s="1">
         <v>25</v>
       </c>
-      <c r="C29" s="1">
-        <f>_xlfn.XLOOKUP(D29,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C29" s="1" t="str">
+        <f>IF(D29="","",_xlfn.XLOOKUP(D29,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D29" s="23"/>
       <c r="E29" s="2" t="str">
@@ -9530,9 +9519,9 @@
       <c r="B30" s="1">
         <v>26</v>
       </c>
-      <c r="C30" s="1">
-        <f>_xlfn.XLOOKUP(D30,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C30" s="1" t="str">
+        <f>IF(D30="","",_xlfn.XLOOKUP(D30,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D30" s="23"/>
       <c r="E30" s="2" t="str">
@@ -9546,20 +9535,16 @@
       </c>
       <c r="K30" s="12">
         <f>K6-K24</f>
-        <v>239000</v>
-      </c>
-      <c r="L30" s="47">
-        <f>485400-K30</f>
-        <v>246400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="2:18">
       <c r="B31" s="1">
         <v>27</v>
       </c>
-      <c r="C31" s="1">
-        <f>_xlfn.XLOOKUP(D31,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C31" s="1" t="str">
+        <f>IF(D31="","",_xlfn.XLOOKUP(D31,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D31" s="23"/>
       <c r="E31" s="2" t="str">
@@ -9573,9 +9558,9 @@
       <c r="B32" s="1">
         <v>28</v>
       </c>
-      <c r="C32" s="1">
-        <f>_xlfn.XLOOKUP(D32,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C32" s="1" t="str">
+        <f>IF(D32="","",_xlfn.XLOOKUP(D32,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D32" s="23"/>
       <c r="E32" s="2" t="str">
@@ -9589,9 +9574,9 @@
       <c r="B33" s="1">
         <v>29</v>
       </c>
-      <c r="C33" s="1">
-        <f>_xlfn.XLOOKUP(D33,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C33" s="1" t="str">
+        <f>IF(D33="","",_xlfn.XLOOKUP(D33,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D33" s="23"/>
       <c r="E33" s="2" t="str">
@@ -9605,9 +9590,9 @@
       <c r="B34" s="1">
         <v>30</v>
       </c>
-      <c r="C34" s="1">
-        <f>_xlfn.XLOOKUP(D34,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C34" s="1" t="str">
+        <f>IF(D34="","",_xlfn.XLOOKUP(D34,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D34" s="23"/>
       <c r="E34" s="2" t="str">
@@ -9621,9 +9606,9 @@
       <c r="B35" s="1">
         <v>31</v>
       </c>
-      <c r="C35" s="1">
-        <f>_xlfn.XLOOKUP(D35,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C35" s="1" t="str">
+        <f>IF(D35="","",_xlfn.XLOOKUP(D35,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D35" s="23"/>
       <c r="E35" s="2" t="str">
@@ -9635,9 +9620,9 @@
       <c r="B36" s="1">
         <v>32</v>
       </c>
-      <c r="C36" s="1">
-        <f>_xlfn.XLOOKUP(D36,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C36" s="1" t="str">
+        <f>IF(D36="","",_xlfn.XLOOKUP(D36,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D36" s="23"/>
       <c r="E36" s="2" t="str">
@@ -9649,9 +9634,9 @@
       <c r="B37" s="1">
         <v>33</v>
       </c>
-      <c r="C37" s="1">
-        <f>_xlfn.XLOOKUP(D37,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C37" s="1" t="str">
+        <f>IF(D37="","",_xlfn.XLOOKUP(D37,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D37" s="23"/>
       <c r="E37" s="2" t="str">
@@ -9663,9 +9648,9 @@
       <c r="B38" s="1">
         <v>34</v>
       </c>
-      <c r="C38" s="1">
-        <f>_xlfn.XLOOKUP(D38,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C38" s="1" t="str">
+        <f>IF(D38="","",_xlfn.XLOOKUP(D38,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D38" s="23"/>
       <c r="E38" s="2" t="str">
@@ -9677,9 +9662,9 @@
       <c r="B39" s="1">
         <v>35</v>
       </c>
-      <c r="C39" s="1">
-        <f>_xlfn.XLOOKUP(D39,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C39" s="1" t="str">
+        <f>IF(D39="","",_xlfn.XLOOKUP(D39,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D39" s="23"/>
       <c r="E39" s="2" t="str">
@@ -9691,9 +9676,9 @@
       <c r="B40" s="1">
         <v>36</v>
       </c>
-      <c r="C40" s="1">
-        <f>_xlfn.XLOOKUP(D40,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C40" s="1" t="str">
+        <f>IF(D40="","",_xlfn.XLOOKUP(D40,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D40" s="23"/>
       <c r="E40" s="2" t="str">
@@ -9705,9 +9690,9 @@
       <c r="B41" s="1">
         <v>37</v>
       </c>
-      <c r="C41" s="1">
-        <f>_xlfn.XLOOKUP(D41,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C41" s="1" t="str">
+        <f>IF(D41="","",_xlfn.XLOOKUP(D41,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D41" s="23"/>
       <c r="E41" s="2" t="str">
@@ -9719,9 +9704,9 @@
       <c r="B42" s="1">
         <v>38</v>
       </c>
-      <c r="C42" s="1">
-        <f>_xlfn.XLOOKUP(D42,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C42" s="1" t="str">
+        <f>IF(D42="","",_xlfn.XLOOKUP(D42,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D42" s="23"/>
       <c r="E42" s="2" t="str">
@@ -9733,9 +9718,9 @@
       <c r="B43" s="1">
         <v>39</v>
       </c>
-      <c r="C43" s="1">
-        <f>_xlfn.XLOOKUP(D43,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C43" s="1" t="str">
+        <f>IF(D43="","",_xlfn.XLOOKUP(D43,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D43" s="23"/>
       <c r="E43" s="2" t="str">
@@ -9747,9 +9732,9 @@
       <c r="B44" s="1">
         <v>40</v>
       </c>
-      <c r="C44" s="1">
-        <f>_xlfn.XLOOKUP(D44,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C44" s="1" t="str">
+        <f>IF(D44="","",_xlfn.XLOOKUP(D44,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D44" s="23"/>
       <c r="E44" s="2" t="str">
@@ -9761,9 +9746,9 @@
       <c r="B45" s="1">
         <v>41</v>
       </c>
-      <c r="C45" s="1">
-        <f>_xlfn.XLOOKUP(D45,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C45" s="1" t="str">
+        <f>IF(D45="","",_xlfn.XLOOKUP(D45,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D45" s="23"/>
       <c r="E45" s="2" t="str">
@@ -9775,9 +9760,9 @@
       <c r="B46" s="1">
         <v>42</v>
       </c>
-      <c r="C46" s="1">
-        <f>_xlfn.XLOOKUP(D46,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C46" s="1" t="str">
+        <f>IF(D46="","",_xlfn.XLOOKUP(D46,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D46" s="23"/>
       <c r="E46" s="2" t="str">
@@ -9789,9 +9774,9 @@
       <c r="B47" s="1">
         <v>43</v>
       </c>
-      <c r="C47" s="1">
-        <f>_xlfn.XLOOKUP(D47,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C47" s="1" t="str">
+        <f>IF(D47="","",_xlfn.XLOOKUP(D47,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D47" s="23"/>
       <c r="E47" s="2" t="str">
@@ -9803,9 +9788,9 @@
       <c r="B48" s="1">
         <v>44</v>
       </c>
-      <c r="C48" s="1">
-        <f>_xlfn.XLOOKUP(D48,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C48" s="1" t="str">
+        <f>IF(D48="","",_xlfn.XLOOKUP(D48,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D48" s="23"/>
       <c r="E48" s="2" t="str">
@@ -9817,9 +9802,9 @@
       <c r="B49" s="1">
         <v>45</v>
       </c>
-      <c r="C49" s="1">
-        <f>_xlfn.XLOOKUP(D49,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C49" s="1" t="str">
+        <f>IF(D49="","",_xlfn.XLOOKUP(D49,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D49" s="23"/>
       <c r="E49" s="2" t="str">
@@ -9831,9 +9816,9 @@
       <c r="B50" s="1">
         <v>46</v>
       </c>
-      <c r="C50" s="1">
-        <f>_xlfn.XLOOKUP(D50,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C50" s="1" t="str">
+        <f>IF(D50="","",_xlfn.XLOOKUP(D50,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D50" s="23"/>
       <c r="E50" s="2" t="str">
@@ -9845,9 +9830,9 @@
       <c r="B51" s="1">
         <v>47</v>
       </c>
-      <c r="C51" s="1">
-        <f>_xlfn.XLOOKUP(D51,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C51" s="1" t="str">
+        <f>IF(D51="","",_xlfn.XLOOKUP(D51,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D51" s="23"/>
       <c r="E51" s="2" t="str">
@@ -9859,9 +9844,9 @@
       <c r="B52" s="1">
         <v>48</v>
       </c>
-      <c r="C52" s="1">
-        <f>_xlfn.XLOOKUP(D52,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C52" s="1" t="str">
+        <f>IF(D52="","",_xlfn.XLOOKUP(D52,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D52" s="23"/>
       <c r="E52" s="2" t="str">
@@ -9873,9 +9858,9 @@
       <c r="B53" s="1">
         <v>49</v>
       </c>
-      <c r="C53" s="1">
-        <f>_xlfn.XLOOKUP(D53,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C53" s="1" t="str">
+        <f>IF(D53="","",_xlfn.XLOOKUP(D53,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D53" s="23"/>
       <c r="E53" s="2" t="str">
@@ -9887,9 +9872,9 @@
       <c r="B54" s="1">
         <v>50</v>
       </c>
-      <c r="C54" s="1">
-        <f>_xlfn.XLOOKUP(D54,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C54" s="1" t="str">
+        <f>IF(D54="","",_xlfn.XLOOKUP(D54,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D54" s="23"/>
       <c r="E54" s="2" t="str">
@@ -9901,9 +9886,9 @@
       <c r="B55" s="1">
         <v>51</v>
       </c>
-      <c r="C55" s="1">
-        <f>_xlfn.XLOOKUP(D55,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C55" s="1" t="str">
+        <f>IF(D55="","",_xlfn.XLOOKUP(D55,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D55" s="23"/>
       <c r="E55" s="2" t="str">
@@ -9915,9 +9900,9 @@
       <c r="B56" s="1">
         <v>52</v>
       </c>
-      <c r="C56" s="1">
-        <f>_xlfn.XLOOKUP(D56,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C56" s="1" t="str">
+        <f>IF(D56="","",_xlfn.XLOOKUP(D56,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D56" s="23"/>
       <c r="E56" s="2" t="str">
@@ -9929,9 +9914,9 @@
       <c r="B57" s="1">
         <v>53</v>
       </c>
-      <c r="C57" s="1">
-        <f>_xlfn.XLOOKUP(D57,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C57" s="1" t="str">
+        <f>IF(D57="","",_xlfn.XLOOKUP(D57,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D57" s="23"/>
       <c r="E57" s="2" t="str">
@@ -9943,9 +9928,9 @@
       <c r="B58" s="1">
         <v>54</v>
       </c>
-      <c r="C58" s="1">
-        <f>_xlfn.XLOOKUP(D58,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C58" s="1" t="str">
+        <f>IF(D58="","",_xlfn.XLOOKUP(D58,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D58" s="23"/>
       <c r="E58" s="2" t="str">
@@ -9957,9 +9942,9 @@
       <c r="B59" s="1">
         <v>55</v>
       </c>
-      <c r="C59" s="1">
-        <f>_xlfn.XLOOKUP(D59,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C59" s="1" t="str">
+        <f>IF(D59="","",_xlfn.XLOOKUP(D59,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D59" s="23"/>
       <c r="E59" s="2" t="str">
@@ -9971,9 +9956,9 @@
       <c r="B60" s="1">
         <v>56</v>
       </c>
-      <c r="C60" s="1">
-        <f>_xlfn.XLOOKUP(D60,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C60" s="1" t="str">
+        <f>IF(D60="","",_xlfn.XLOOKUP(D60,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D60" s="23"/>
       <c r="E60" s="2" t="str">
@@ -9985,9 +9970,9 @@
       <c r="B61" s="1">
         <v>57</v>
       </c>
-      <c r="C61" s="1">
-        <f>_xlfn.XLOOKUP(D61,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C61" s="1" t="str">
+        <f>IF(D61="","",_xlfn.XLOOKUP(D61,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D61" s="23"/>
       <c r="E61" s="2" t="str">
@@ -9999,9 +9984,9 @@
       <c r="B62" s="1">
         <v>58</v>
       </c>
-      <c r="C62" s="1">
-        <f>_xlfn.XLOOKUP(D62,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C62" s="1" t="str">
+        <f>IF(D62="","",_xlfn.XLOOKUP(D62,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D62" s="23"/>
       <c r="E62" s="2" t="str">
@@ -10013,9 +9998,9 @@
       <c r="B63" s="1">
         <v>59</v>
       </c>
-      <c r="C63" s="1">
-        <f>_xlfn.XLOOKUP(D63,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C63" s="1" t="str">
+        <f>IF(D63="","",_xlfn.XLOOKUP(D63,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D63" s="23"/>
       <c r="E63" s="2" t="str">
@@ -10027,9 +10012,9 @@
       <c r="B64" s="1">
         <v>60</v>
       </c>
-      <c r="C64" s="1">
-        <f>_xlfn.XLOOKUP(D64,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C64" s="1" t="str">
+        <f>IF(D64="","",_xlfn.XLOOKUP(D64,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D64" s="23"/>
       <c r="E64" s="2" t="str">
@@ -10041,9 +10026,9 @@
       <c r="B65" s="1">
         <v>61</v>
       </c>
-      <c r="C65" s="1">
-        <f>_xlfn.XLOOKUP(D65,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C65" s="1" t="str">
+        <f>IF(D65="","",_xlfn.XLOOKUP(D65,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D65" s="23"/>
       <c r="E65" s="2" t="str">
@@ -10055,9 +10040,9 @@
       <c r="B66" s="1">
         <v>62</v>
       </c>
-      <c r="C66" s="1">
-        <f>_xlfn.XLOOKUP(D66,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C66" s="1" t="str">
+        <f>IF(D66="","",_xlfn.XLOOKUP(D66,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D66" s="23"/>
       <c r="E66" s="2" t="str">
@@ -10069,9 +10054,9 @@
       <c r="B67" s="1">
         <v>63</v>
       </c>
-      <c r="C67" s="1">
-        <f>_xlfn.XLOOKUP(D67,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C67" s="1" t="str">
+        <f>IF(D67="","",_xlfn.XLOOKUP(D67,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D67" s="23"/>
       <c r="E67" s="2" t="str">
@@ -10083,9 +10068,9 @@
       <c r="B68" s="1">
         <v>64</v>
       </c>
-      <c r="C68" s="1">
-        <f>_xlfn.XLOOKUP(D68,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C68" s="1" t="str">
+        <f>IF(D68="","",_xlfn.XLOOKUP(D68,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D68" s="23"/>
       <c r="E68" s="2" t="str">
@@ -10097,9 +10082,9 @@
       <c r="B69" s="1">
         <v>65</v>
       </c>
-      <c r="C69" s="1">
-        <f>_xlfn.XLOOKUP(D69,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C69" s="1" t="str">
+        <f>IF(D69="","",_xlfn.XLOOKUP(D69,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D69" s="23"/>
       <c r="E69" s="2" t="str">
@@ -10111,9 +10096,9 @@
       <c r="B70" s="1">
         <v>66</v>
       </c>
-      <c r="C70" s="1">
-        <f>_xlfn.XLOOKUP(D70,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C70" s="1" t="str">
+        <f>IF(D70="","",_xlfn.XLOOKUP(D70,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D70" s="23"/>
       <c r="E70" s="2" t="str">
@@ -10125,9 +10110,9 @@
       <c r="B71" s="1">
         <v>67</v>
       </c>
-      <c r="C71" s="1">
-        <f>_xlfn.XLOOKUP(D71,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C71" s="1" t="str">
+        <f>IF(D71="","",_xlfn.XLOOKUP(D71,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D71" s="23"/>
       <c r="E71" s="2" t="str">
@@ -10139,9 +10124,9 @@
       <c r="B72" s="1">
         <v>68</v>
       </c>
-      <c r="C72" s="1">
-        <f>_xlfn.XLOOKUP(D72,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C72" s="1" t="str">
+        <f>IF(D72="","",_xlfn.XLOOKUP(D72,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D72" s="23"/>
       <c r="E72" s="2" t="str">
@@ -10153,9 +10138,9 @@
       <c r="B73" s="1">
         <v>69</v>
       </c>
-      <c r="C73" s="1">
-        <f>_xlfn.XLOOKUP(D73,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C73" s="1" t="str">
+        <f>IF(D73="","",_xlfn.XLOOKUP(D73,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D73" s="23"/>
       <c r="E73" s="2" t="str">
@@ -10167,9 +10152,9 @@
       <c r="B74" s="1">
         <v>70</v>
       </c>
-      <c r="C74" s="1">
-        <f>_xlfn.XLOOKUP(D74,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C74" s="1" t="str">
+        <f>IF(D74="","",_xlfn.XLOOKUP(D74,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D74" s="23"/>
       <c r="E74" s="2" t="str">
@@ -10181,9 +10166,9 @@
       <c r="B75" s="1">
         <v>71</v>
       </c>
-      <c r="C75" s="1">
-        <f>_xlfn.XLOOKUP(D75,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C75" s="1" t="str">
+        <f>IF(D75="","",_xlfn.XLOOKUP(D75,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D75" s="23"/>
       <c r="E75" s="2" t="str">
@@ -10195,9 +10180,9 @@
       <c r="B76" s="1">
         <v>72</v>
       </c>
-      <c r="C76" s="1">
-        <f>_xlfn.XLOOKUP(D76,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C76" s="1" t="str">
+        <f>IF(D76="","",_xlfn.XLOOKUP(D76,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D76" s="23"/>
       <c r="E76" s="2" t="str">
@@ -10209,9 +10194,9 @@
       <c r="B77" s="1">
         <v>73</v>
       </c>
-      <c r="C77" s="1">
-        <f>_xlfn.XLOOKUP(D77,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C77" s="1" t="str">
+        <f>IF(D77="","",_xlfn.XLOOKUP(D77,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D77" s="23"/>
       <c r="E77" s="2" t="str">
@@ -10223,9 +10208,9 @@
       <c r="B78" s="1">
         <v>74</v>
       </c>
-      <c r="C78" s="1">
-        <f>_xlfn.XLOOKUP(D78,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C78" s="1" t="str">
+        <f>IF(D78="","",_xlfn.XLOOKUP(D78,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D78" s="23"/>
       <c r="E78" s="2" t="str">
@@ -10237,9 +10222,9 @@
       <c r="B79" s="1">
         <v>75</v>
       </c>
-      <c r="C79" s="1">
-        <f>_xlfn.XLOOKUP(D79,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C79" s="1" t="str">
+        <f>IF(D79="","",_xlfn.XLOOKUP(D79,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D79" s="23"/>
       <c r="E79" s="2" t="str">
@@ -10251,9 +10236,9 @@
       <c r="B80" s="1">
         <v>76</v>
       </c>
-      <c r="C80" s="1">
-        <f>_xlfn.XLOOKUP(D80,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C80" s="1" t="str">
+        <f>IF(D80="","",_xlfn.XLOOKUP(D80,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D80" s="23"/>
       <c r="E80" s="2" t="str">
@@ -10265,9 +10250,9 @@
       <c r="B81" s="1">
         <v>77</v>
       </c>
-      <c r="C81" s="1">
-        <f>_xlfn.XLOOKUP(D81,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C81" s="1" t="str">
+        <f>IF(D81="","",_xlfn.XLOOKUP(D81,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D81" s="23"/>
       <c r="E81" s="2" t="str">
@@ -10279,9 +10264,9 @@
       <c r="B82" s="1">
         <v>78</v>
       </c>
-      <c r="C82" s="1">
-        <f>_xlfn.XLOOKUP(D82,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C82" s="1" t="str">
+        <f>IF(D82="","",_xlfn.XLOOKUP(D82,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D82" s="23"/>
       <c r="E82" s="2" t="str">
@@ -10293,9 +10278,9 @@
       <c r="B83" s="1">
         <v>79</v>
       </c>
-      <c r="C83" s="1">
-        <f>_xlfn.XLOOKUP(D83,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C83" s="1" t="str">
+        <f>IF(D83="","",_xlfn.XLOOKUP(D83,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D83" s="23"/>
       <c r="E83" s="2" t="str">
@@ -10307,9 +10292,9 @@
       <c r="B84" s="1">
         <v>80</v>
       </c>
-      <c r="C84" s="1">
-        <f>_xlfn.XLOOKUP(D84,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C84" s="1" t="str">
+        <f>IF(D84="","",_xlfn.XLOOKUP(D84,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D84" s="23"/>
       <c r="E84" s="2" t="str">
@@ -10321,9 +10306,9 @@
       <c r="B85" s="1">
         <v>81</v>
       </c>
-      <c r="C85" s="1">
-        <f>_xlfn.XLOOKUP(D85,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C85" s="1" t="str">
+        <f>IF(D85="","",_xlfn.XLOOKUP(D85,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D85" s="23"/>
       <c r="E85" s="2" t="str">
@@ -10335,9 +10320,9 @@
       <c r="B86" s="1">
         <v>82</v>
       </c>
-      <c r="C86" s="1">
-        <f>_xlfn.XLOOKUP(D86,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C86" s="1" t="str">
+        <f>IF(D86="","",_xlfn.XLOOKUP(D86,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D86" s="23"/>
       <c r="E86" s="2" t="str">
@@ -10349,9 +10334,9 @@
       <c r="B87" s="1">
         <v>83</v>
       </c>
-      <c r="C87" s="1">
-        <f>_xlfn.XLOOKUP(D87,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C87" s="1" t="str">
+        <f>IF(D87="","",_xlfn.XLOOKUP(D87,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D87" s="23"/>
       <c r="E87" s="2" t="str">
@@ -10363,9 +10348,9 @@
       <c r="B88" s="1">
         <v>84</v>
       </c>
-      <c r="C88" s="1">
-        <f>_xlfn.XLOOKUP(D88,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C88" s="1" t="str">
+        <f>IF(D88="","",_xlfn.XLOOKUP(D88,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D88" s="23"/>
       <c r="E88" s="2" t="str">
@@ -10377,9 +10362,9 @@
       <c r="B89" s="1">
         <v>85</v>
       </c>
-      <c r="C89" s="1">
-        <f>_xlfn.XLOOKUP(D89,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C89" s="1" t="str">
+        <f>IF(D89="","",_xlfn.XLOOKUP(D89,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D89" s="23"/>
       <c r="E89" s="2" t="str">
@@ -10391,9 +10376,9 @@
       <c r="B90" s="1">
         <v>86</v>
       </c>
-      <c r="C90" s="1">
-        <f>_xlfn.XLOOKUP(D90,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C90" s="1" t="str">
+        <f>IF(D90="","",_xlfn.XLOOKUP(D90,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D90" s="23"/>
       <c r="E90" s="2" t="str">
@@ -10405,9 +10390,9 @@
       <c r="B91" s="1">
         <v>87</v>
       </c>
-      <c r="C91" s="1">
-        <f>_xlfn.XLOOKUP(D91,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C91" s="1" t="str">
+        <f>IF(D91="","",_xlfn.XLOOKUP(D91,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D91" s="23"/>
       <c r="E91" s="2" t="str">
@@ -10419,9 +10404,9 @@
       <c r="B92" s="1">
         <v>88</v>
       </c>
-      <c r="C92" s="1">
-        <f>_xlfn.XLOOKUP(D92,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C92" s="1" t="str">
+        <f>IF(D92="","",_xlfn.XLOOKUP(D92,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D92" s="23"/>
       <c r="E92" s="2" t="str">
@@ -10433,9 +10418,9 @@
       <c r="B93" s="1">
         <v>89</v>
       </c>
-      <c r="C93" s="1">
-        <f>_xlfn.XLOOKUP(D93,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C93" s="1" t="str">
+        <f>IF(D93="","",_xlfn.XLOOKUP(D93,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D93" s="23"/>
       <c r="E93" s="2" t="str">
@@ -10447,9 +10432,9 @@
       <c r="B94" s="1">
         <v>90</v>
       </c>
-      <c r="C94" s="1">
-        <f>_xlfn.XLOOKUP(D94,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C94" s="1" t="str">
+        <f>IF(D94="","",_xlfn.XLOOKUP(D94,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D94" s="23"/>
       <c r="E94" s="2" t="str">
@@ -10461,9 +10446,9 @@
       <c r="B95" s="1">
         <v>91</v>
       </c>
-      <c r="C95" s="1">
-        <f>_xlfn.XLOOKUP(D95,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C95" s="1" t="str">
+        <f>IF(D95="","",_xlfn.XLOOKUP(D95,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D95" s="23"/>
       <c r="E95" s="2" t="str">
@@ -10475,9 +10460,9 @@
       <c r="B96" s="1">
         <v>92</v>
       </c>
-      <c r="C96" s="1">
-        <f>_xlfn.XLOOKUP(D96,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C96" s="1" t="str">
+        <f>IF(D96="","",_xlfn.XLOOKUP(D96,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D96" s="23"/>
       <c r="E96" s="2" t="str">
@@ -10489,9 +10474,9 @@
       <c r="B97" s="1">
         <v>93</v>
       </c>
-      <c r="C97" s="1">
-        <f>_xlfn.XLOOKUP(D97,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C97" s="1" t="str">
+        <f>IF(D97="","",_xlfn.XLOOKUP(D97,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D97" s="23"/>
       <c r="E97" s="2" t="str">
@@ -10503,9 +10488,9 @@
       <c r="B98" s="1">
         <v>94</v>
       </c>
-      <c r="C98" s="1">
-        <f>_xlfn.XLOOKUP(D98,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C98" s="1" t="str">
+        <f>IF(D98="","",_xlfn.XLOOKUP(D98,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D98" s="23"/>
       <c r="E98" s="2" t="str">
@@ -10517,9 +10502,9 @@
       <c r="B99" s="1">
         <v>95</v>
       </c>
-      <c r="C99" s="1">
-        <f>_xlfn.XLOOKUP(D99,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C99" s="1" t="str">
+        <f>IF(D99="","",_xlfn.XLOOKUP(D99,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D99" s="23"/>
       <c r="E99" s="2" t="str">
@@ -10531,9 +10516,9 @@
       <c r="B100" s="1">
         <v>96</v>
       </c>
-      <c r="C100" s="1">
-        <f>_xlfn.XLOOKUP(D100,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C100" s="1" t="str">
+        <f>IF(D100="","",_xlfn.XLOOKUP(D100,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D100" s="23"/>
       <c r="E100" s="2" t="str">
@@ -10545,9 +10530,9 @@
       <c r="B101" s="1">
         <v>97</v>
       </c>
-      <c r="C101" s="1">
-        <f>_xlfn.XLOOKUP(D101,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C101" s="1" t="str">
+        <f>IF(D101="","",_xlfn.XLOOKUP(D101,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D101" s="23"/>
       <c r="E101" s="2" t="str">
@@ -10559,9 +10544,9 @@
       <c r="B102" s="1">
         <v>98</v>
       </c>
-      <c r="C102" s="1">
-        <f>_xlfn.XLOOKUP(D102,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C102" s="1" t="str">
+        <f>IF(D102="","",_xlfn.XLOOKUP(D102,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D102" s="23"/>
       <c r="E102" s="2" t="str">
@@ -10573,9 +10558,9 @@
       <c r="B103" s="1">
         <v>99</v>
       </c>
-      <c r="C103" s="1">
-        <f>_xlfn.XLOOKUP(D103,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C103" s="1" t="str">
+        <f>IF(D103="","",_xlfn.XLOOKUP(D103,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D103" s="23"/>
       <c r="E103" s="2" t="str">
@@ -10587,9 +10572,9 @@
       <c r="B104" s="1">
         <v>100</v>
       </c>
-      <c r="C104" s="1">
-        <f>_xlfn.XLOOKUP(D104,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C104" s="1" t="str">
+        <f>IF(D104="","",_xlfn.XLOOKUP(D104,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D104" s="23"/>
       <c r="E104" s="2" t="str">
@@ -10601,9 +10586,9 @@
       <c r="B105" s="1">
         <v>101</v>
       </c>
-      <c r="C105" s="1">
-        <f>_xlfn.XLOOKUP(D105,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C105" s="1" t="str">
+        <f>IF(D105="","",_xlfn.XLOOKUP(D105,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D105" s="23"/>
       <c r="E105" s="2" t="str">
@@ -10615,9 +10600,9 @@
       <c r="B106" s="1">
         <v>102</v>
       </c>
-      <c r="C106" s="1">
-        <f>_xlfn.XLOOKUP(D106,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C106" s="1" t="str">
+        <f>IF(D106="","",_xlfn.XLOOKUP(D106,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D106" s="23"/>
       <c r="E106" s="2" t="str">
@@ -10629,9 +10614,9 @@
       <c r="B107" s="1">
         <v>103</v>
       </c>
-      <c r="C107" s="1">
-        <f>_xlfn.XLOOKUP(D107,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C107" s="1" t="str">
+        <f>IF(D107="","",_xlfn.XLOOKUP(D107,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D107" s="23"/>
       <c r="E107" s="2" t="str">
@@ -10643,9 +10628,9 @@
       <c r="B108" s="1">
         <v>104</v>
       </c>
-      <c r="C108" s="1">
-        <f>_xlfn.XLOOKUP(D108,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C108" s="1" t="str">
+        <f>IF(D108="","",_xlfn.XLOOKUP(D108,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D108" s="23"/>
       <c r="E108" s="2" t="str">
@@ -10657,9 +10642,9 @@
       <c r="B109" s="1">
         <v>105</v>
       </c>
-      <c r="C109" s="1">
-        <f>_xlfn.XLOOKUP(D109,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C109" s="1" t="str">
+        <f>IF(D109="","",_xlfn.XLOOKUP(D109,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D109" s="23"/>
       <c r="E109" s="2" t="str">
@@ -10671,9 +10656,9 @@
       <c r="B110" s="1">
         <v>106</v>
       </c>
-      <c r="C110" s="1">
-        <f>_xlfn.XLOOKUP(D110,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C110" s="1" t="str">
+        <f>IF(D110="","",_xlfn.XLOOKUP(D110,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D110" s="23"/>
       <c r="E110" s="2" t="str">
@@ -10685,9 +10670,9 @@
       <c r="B111" s="1">
         <v>107</v>
       </c>
-      <c r="C111" s="1">
-        <f>_xlfn.XLOOKUP(D111,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C111" s="1" t="str">
+        <f>IF(D111="","",_xlfn.XLOOKUP(D111,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D111" s="23"/>
       <c r="E111" s="2" t="str">
@@ -10699,9 +10684,9 @@
       <c r="B112" s="1">
         <v>108</v>
       </c>
-      <c r="C112" s="1">
-        <f>_xlfn.XLOOKUP(D112,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C112" s="1" t="str">
+        <f>IF(D112="","",_xlfn.XLOOKUP(D112,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D112" s="23"/>
       <c r="E112" s="2" t="str">
@@ -10713,9 +10698,9 @@
       <c r="B113" s="1">
         <v>109</v>
       </c>
-      <c r="C113" s="1">
-        <f>_xlfn.XLOOKUP(D113,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C113" s="1" t="str">
+        <f>IF(D113="","",_xlfn.XLOOKUP(D113,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D113" s="23"/>
       <c r="E113" s="2" t="str">
@@ -10727,9 +10712,9 @@
       <c r="B114" s="1">
         <v>110</v>
       </c>
-      <c r="C114" s="1">
-        <f>_xlfn.XLOOKUP(D114,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C114" s="1" t="str">
+        <f>IF(D114="","",_xlfn.XLOOKUP(D114,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D114" s="23"/>
       <c r="E114" s="2" t="str">
@@ -10741,9 +10726,9 @@
       <c r="B115" s="1">
         <v>111</v>
       </c>
-      <c r="C115" s="1">
-        <f>_xlfn.XLOOKUP(D115,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C115" s="1" t="str">
+        <f>IF(D115="","",_xlfn.XLOOKUP(D115,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D115" s="23"/>
       <c r="E115" s="2" t="str">
@@ -10755,9 +10740,9 @@
       <c r="B116" s="1">
         <v>112</v>
       </c>
-      <c r="C116" s="1">
-        <f>_xlfn.XLOOKUP(D116,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C116" s="1" t="str">
+        <f>IF(D116="","",_xlfn.XLOOKUP(D116,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D116" s="23"/>
       <c r="E116" s="2" t="str">
@@ -10769,9 +10754,9 @@
       <c r="B117" s="1">
         <v>113</v>
       </c>
-      <c r="C117" s="1">
-        <f>_xlfn.XLOOKUP(D117,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C117" s="1" t="str">
+        <f>IF(D117="","",_xlfn.XLOOKUP(D117,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D117" s="23"/>
       <c r="E117" s="2" t="str">
@@ -10783,9 +10768,9 @@
       <c r="B118" s="1">
         <v>114</v>
       </c>
-      <c r="C118" s="1">
-        <f>_xlfn.XLOOKUP(D118,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C118" s="1" t="str">
+        <f>IF(D118="","",_xlfn.XLOOKUP(D118,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D118" s="23"/>
       <c r="E118" s="2" t="str">
@@ -10797,9 +10782,9 @@
       <c r="B119" s="1">
         <v>115</v>
       </c>
-      <c r="C119" s="1">
-        <f>_xlfn.XLOOKUP(D119,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C119" s="1" t="str">
+        <f>IF(D119="","",_xlfn.XLOOKUP(D119,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D119" s="23"/>
       <c r="E119" s="2" t="str">
@@ -10811,9 +10796,9 @@
       <c r="B120" s="1">
         <v>116</v>
       </c>
-      <c r="C120" s="1">
-        <f>_xlfn.XLOOKUP(D120,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C120" s="1" t="str">
+        <f>IF(D120="","",_xlfn.XLOOKUP(D120,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D120" s="23"/>
       <c r="E120" s="2" t="str">
@@ -10825,9 +10810,9 @@
       <c r="B121" s="1">
         <v>117</v>
       </c>
-      <c r="C121" s="1">
-        <f>_xlfn.XLOOKUP(D121,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C121" s="1" t="str">
+        <f>IF(D121="","",_xlfn.XLOOKUP(D121,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D121" s="23"/>
       <c r="E121" s="2" t="str">
@@ -10839,9 +10824,9 @@
       <c r="B122" s="1">
         <v>118</v>
       </c>
-      <c r="C122" s="1">
-        <f>_xlfn.XLOOKUP(D122,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C122" s="1" t="str">
+        <f>IF(D122="","",_xlfn.XLOOKUP(D122,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D122" s="23"/>
       <c r="E122" s="2" t="str">
@@ -10853,9 +10838,9 @@
       <c r="B123" s="1">
         <v>119</v>
       </c>
-      <c r="C123" s="1">
-        <f>_xlfn.XLOOKUP(D123,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C123" s="1" t="str">
+        <f>IF(D123="","",_xlfn.XLOOKUP(D123,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D123" s="23"/>
       <c r="E123" s="2" t="str">
@@ -10867,9 +10852,9 @@
       <c r="B124" s="1">
         <v>120</v>
       </c>
-      <c r="C124" s="1">
-        <f>_xlfn.XLOOKUP(D124,'Global ID'!C:C,'Global ID'!B:B,"")</f>
-        <v>0</v>
+      <c r="C124" s="1" t="str">
+        <f>IF(D124="","",_xlfn.XLOOKUP(D124,'Global ID'!$C$1:$C$2000,'Global ID'!$B$1:$B$2000,,0))</f>
+        <v/>
       </c>
       <c r="D124" s="23"/>
       <c r="E124" s="2" t="str">
@@ -10952,14 +10937,14 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6422ACDB-AD6F-44F4-BFCF-4AA6AE95A6C0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D803447-D6A8-4128-976A-83F700697131}">
   <dimension ref="A1:Q8"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="2" max="2" width="30.58203125" style="48" customWidth="1"/>
-    <col min="3" max="3" width="4.75" style="48" customWidth="1"/>
-    <col min="4" max="4" width="30.58203125" style="48" customWidth="1"/>
-    <col min="5" max="10" width="8.6640625" style="48"/>
+    <col min="2" max="2" width="30.58203125" style="52" customWidth="1"/>
+    <col min="3" max="3" width="4.75" style="52" customWidth="1"/>
+    <col min="4" max="4" width="30.58203125" style="52" customWidth="1"/>
+    <col min="5" max="10" width="8.6640625" style="52"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18.5">
@@ -10968,11 +10953,11 @@
       </c>
     </row>
     <row r="4" spans="1:17" ht="16">
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="53" t="s">
+        <v>2628</v>
+      </c>
+      <c r="D4" s="53" t="s">
         <v>2629</v>
-      </c>
-      <c r="D4" s="49" t="s">
-        <v>2628</v>
       </c>
       <c r="Q4" s="46"/>
     </row>
@@ -10980,7 +10965,6 @@
       <c r="D8" s="45"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>